<commit_message>
MMSC + MM01 (Smart Wait Exp) + Compare Stock
</commit_message>
<xml_diff>
--- a/config/Material_Template_MM01.xlsx
+++ b/config/Material_Template_MM01.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6800"/>
+    <workbookView windowWidth="19200" windowHeight="6200"/>
   </bookViews>
   <sheets>
     <sheet name="Material List" sheetId="1" r:id="rId1"/>
@@ -758,7 +758,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -779,6 +779,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1175,7 +1178,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="5">
-        <v>315332</v>
+        <v>410809</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="6"/>
@@ -1185,9 +1188,7 @@
       <c r="A5" s="4">
         <v>2</v>
       </c>
-      <c r="B5" s="7">
-        <v>315001</v>
-      </c>
+      <c r="B5" s="7"/>
       <c r="C5" s="5"/>
       <c r="D5" s="6"/>
       <c r="E5" s="5"/>
@@ -1196,8 +1197,9 @@
       <c r="A6" s="4">
         <v>3</v>
       </c>
+      <c r="B6" s="8"/>
       <c r="C6" s="7"/>
-      <c r="D6" s="8"/>
+      <c r="D6" s="9"/>
       <c r="E6" s="7"/>
     </row>
     <row r="7" ht="18" customHeight="1" spans="1:5">
@@ -1206,7 +1208,7 @@
       </c>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
-      <c r="D7" s="8"/>
+      <c r="D7" s="9"/>
       <c r="E7" s="7"/>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:5">
@@ -1215,7 +1217,7 @@
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
-      <c r="D8" s="8"/>
+      <c r="D8" s="9"/>
       <c r="E8" s="7"/>
     </row>
     <row r="9" ht="18" customHeight="1" spans="1:5">
@@ -1224,7 +1226,7 @@
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
-      <c r="D9" s="8"/>
+      <c r="D9" s="9"/>
       <c r="E9" s="7"/>
     </row>
     <row r="10" ht="18" customHeight="1" spans="1:5">
@@ -1233,7 +1235,7 @@
       </c>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
-      <c r="D10" s="8"/>
+      <c r="D10" s="9"/>
       <c r="E10" s="7"/>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:5">
@@ -1242,7 +1244,7 @@
       </c>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
-      <c r="D11" s="8"/>
+      <c r="D11" s="9"/>
       <c r="E11" s="7"/>
     </row>
     <row r="12" ht="18" customHeight="1" spans="1:5">
@@ -1251,7 +1253,7 @@
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
-      <c r="D12" s="8"/>
+      <c r="D12" s="9"/>
       <c r="E12" s="7"/>
     </row>
     <row r="13" ht="18" customHeight="1" spans="1:5">
@@ -1260,7 +1262,7 @@
       </c>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
-      <c r="D13" s="8"/>
+      <c r="D13" s="9"/>
       <c r="E13" s="7"/>
     </row>
     <row r="14" ht="18" customHeight="1" spans="1:5">
@@ -1269,7 +1271,7 @@
       </c>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
-      <c r="D14" s="8"/>
+      <c r="D14" s="9"/>
       <c r="E14" s="7"/>
     </row>
     <row r="15" ht="18" customHeight="1" spans="1:5">
@@ -1278,7 +1280,7 @@
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
-      <c r="D15" s="8"/>
+      <c r="D15" s="9"/>
       <c r="E15" s="7"/>
     </row>
     <row r="16" ht="18" customHeight="1" spans="1:5">
@@ -1287,7 +1289,7 @@
       </c>
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
-      <c r="D16" s="8"/>
+      <c r="D16" s="9"/>
       <c r="E16" s="7"/>
     </row>
     <row r="17" ht="18" customHeight="1" spans="1:5">
@@ -1296,7 +1298,7 @@
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
-      <c r="D17" s="8"/>
+      <c r="D17" s="9"/>
       <c r="E17" s="7"/>
     </row>
     <row r="18" ht="18" customHeight="1" spans="1:5">
@@ -1305,7 +1307,7 @@
       </c>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
-      <c r="D18" s="8"/>
+      <c r="D18" s="9"/>
       <c r="E18" s="7"/>
     </row>
     <row r="19" ht="18" customHeight="1" spans="1:5">
@@ -1314,7 +1316,7 @@
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
-      <c r="D19" s="8"/>
+      <c r="D19" s="9"/>
       <c r="E19" s="7"/>
     </row>
     <row r="20" ht="18" customHeight="1" spans="1:5">
@@ -1323,7 +1325,7 @@
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
-      <c r="D20" s="8"/>
+      <c r="D20" s="9"/>
       <c r="E20" s="7"/>
     </row>
     <row r="21" ht="18" customHeight="1" spans="1:5">
@@ -1332,7 +1334,7 @@
       </c>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
-      <c r="D21" s="8"/>
+      <c r="D21" s="9"/>
       <c r="E21" s="7"/>
     </row>
     <row r="22" ht="18" customHeight="1" spans="1:5">
@@ -1341,7 +1343,7 @@
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
-      <c r="D22" s="8"/>
+      <c r="D22" s="9"/>
       <c r="E22" s="7"/>
     </row>
     <row r="23" ht="18" customHeight="1" spans="1:5">
@@ -1350,7 +1352,7 @@
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
-      <c r="D23" s="8"/>
+      <c r="D23" s="9"/>
       <c r="E23" s="7"/>
     </row>
     <row r="24" ht="18" customHeight="1" spans="1:5">
@@ -1359,7 +1361,7 @@
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
-      <c r="D24" s="8"/>
+      <c r="D24" s="9"/>
       <c r="E24" s="7"/>
     </row>
     <row r="25" ht="18" customHeight="1" spans="1:5">
@@ -1368,7 +1370,7 @@
       </c>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
-      <c r="D25" s="8"/>
+      <c r="D25" s="9"/>
       <c r="E25" s="7"/>
     </row>
     <row r="26" ht="18" customHeight="1" spans="1:5">
@@ -1377,7 +1379,7 @@
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
-      <c r="D26" s="8"/>
+      <c r="D26" s="9"/>
       <c r="E26" s="7"/>
     </row>
     <row r="27" ht="18" customHeight="1" spans="1:5">
@@ -1386,7 +1388,7 @@
       </c>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
-      <c r="D27" s="8"/>
+      <c r="D27" s="9"/>
       <c r="E27" s="7"/>
     </row>
     <row r="28" ht="18" customHeight="1" spans="1:5">
@@ -1395,7 +1397,7 @@
       </c>
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
-      <c r="D28" s="8"/>
+      <c r="D28" s="9"/>
       <c r="E28" s="7"/>
     </row>
     <row r="29" ht="18" customHeight="1" spans="1:5">
@@ -1404,7 +1406,7 @@
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
-      <c r="D29" s="8"/>
+      <c r="D29" s="9"/>
       <c r="E29" s="7"/>
     </row>
     <row r="30" ht="18" customHeight="1" spans="1:5">
@@ -1413,11 +1415,11 @@
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>
-      <c r="D30" s="8"/>
+      <c r="D30" s="9"/>
       <c r="E30" s="7"/>
     </row>
     <row r="31" ht="18" customHeight="1" spans="1:5">
-      <c r="A31" s="9" t="s">
+      <c r="A31" s="10" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Maintain Material + Compare Stock Update
</commit_message>
<xml_diff>
--- a/config/Material_Template_MM01.xlsx
+++ b/config/Material_Template_MM01.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6200"/>
+    <workbookView windowWidth="19200" windowHeight="6800"/>
   </bookViews>
   <sheets>
     <sheet name="Material List" sheetId="1" r:id="rId1"/>
@@ -63,7 +63,7 @@
     <numFmt numFmtId="178" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="179" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -99,14 +99,35 @@
       <charset val="134"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <charset val="134"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <charset val="134"/>
     </font>
     <font>
@@ -281,13 +302,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFAFAFA"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFAFAFA"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -628,137 +649,137 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -772,20 +793,19 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1178,248 +1198,246 @@
         <v>1</v>
       </c>
       <c r="B4" s="5">
-        <v>410809</v>
-      </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="5"/>
+        <v>370192</v>
+      </c>
+      <c r="C4" s="6"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="8"/>
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:5">
       <c r="A5" s="4">
         <v>2</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="5"/>
+      <c r="B5" s="5">
+        <v>370194</v>
+      </c>
     </row>
     <row r="6" ht="18" customHeight="1" spans="1:5">
       <c r="A6" s="4">
         <v>3</v>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="7"/>
+      <c r="B6" s="5">
+        <v>370195</v>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1" spans="1:5">
       <c r="A7" s="4">
         <v>4</v>
       </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="7"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="8"/>
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:5">
       <c r="A8" s="4">
         <v>5</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="7"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="8"/>
     </row>
     <row r="9" ht="18" customHeight="1" spans="1:5">
       <c r="A9" s="4">
         <v>6</v>
       </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="7"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="8"/>
     </row>
     <row r="10" ht="18" customHeight="1" spans="1:5">
       <c r="A10" s="4">
         <v>7</v>
       </c>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="7"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="6"/>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:5">
       <c r="A11" s="4">
         <v>8</v>
       </c>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="7"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="6"/>
     </row>
     <row r="12" ht="18" customHeight="1" spans="1:5">
       <c r="A12" s="4">
         <v>9</v>
       </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="7"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="6"/>
     </row>
     <row r="13" ht="18" customHeight="1" spans="1:5">
       <c r="A13" s="4">
         <v>10</v>
       </c>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="7"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="6"/>
     </row>
     <row r="14" ht="18" customHeight="1" spans="1:5">
       <c r="A14" s="4">
         <v>11</v>
       </c>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="7"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="6"/>
     </row>
     <row r="15" ht="18" customHeight="1" spans="1:5">
       <c r="A15" s="4">
         <v>12</v>
       </c>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="7"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="6"/>
     </row>
     <row r="16" ht="18" customHeight="1" spans="1:5">
       <c r="A16" s="4">
         <v>13</v>
       </c>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="7"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="6"/>
     </row>
     <row r="17" ht="18" customHeight="1" spans="1:5">
       <c r="A17" s="4">
         <v>14</v>
       </c>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="7"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="6"/>
     </row>
     <row r="18" ht="18" customHeight="1" spans="1:5">
       <c r="A18" s="4">
         <v>15</v>
       </c>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="7"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="6"/>
     </row>
     <row r="19" ht="18" customHeight="1" spans="1:5">
       <c r="A19" s="4">
         <v>16</v>
       </c>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="7"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="6"/>
     </row>
     <row r="20" ht="18" customHeight="1" spans="1:5">
       <c r="A20" s="4">
         <v>17</v>
       </c>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="7"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="6"/>
     </row>
     <row r="21" ht="18" customHeight="1" spans="1:5">
       <c r="A21" s="4">
         <v>18</v>
       </c>
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="7"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="6"/>
     </row>
     <row r="22" ht="18" customHeight="1" spans="1:5">
       <c r="A22" s="4">
         <v>19</v>
       </c>
-      <c r="B22" s="7"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="7"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="6"/>
     </row>
     <row r="23" ht="18" customHeight="1" spans="1:5">
       <c r="A23" s="4">
         <v>20</v>
       </c>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="7"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="6"/>
     </row>
     <row r="24" ht="18" customHeight="1" spans="1:5">
       <c r="A24" s="4">
         <v>21</v>
       </c>
-      <c r="B24" s="7"/>
-      <c r="C24" s="7"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="7"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="6"/>
     </row>
     <row r="25" ht="18" customHeight="1" spans="1:5">
       <c r="A25" s="4">
         <v>22</v>
       </c>
-      <c r="B25" s="7"/>
-      <c r="C25" s="7"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="7"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="6"/>
     </row>
     <row r="26" ht="18" customHeight="1" spans="1:5">
       <c r="A26" s="4">
         <v>23</v>
       </c>
-      <c r="B26" s="7"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="7"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="6"/>
     </row>
     <row r="27" ht="18" customHeight="1" spans="1:5">
       <c r="A27" s="4">
         <v>24</v>
       </c>
-      <c r="B27" s="7"/>
-      <c r="C27" s="7"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="7"/>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="6"/>
     </row>
     <row r="28" ht="18" customHeight="1" spans="1:5">
       <c r="A28" s="4">
         <v>25</v>
       </c>
-      <c r="B28" s="7"/>
-      <c r="C28" s="7"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="7"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="7"/>
+      <c r="E28" s="6"/>
     </row>
     <row r="29" ht="18" customHeight="1" spans="1:5">
       <c r="A29" s="4">
         <v>26</v>
       </c>
-      <c r="B29" s="7"/>
-      <c r="C29" s="7"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="7"/>
+      <c r="B29" s="6"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="7"/>
+      <c r="E29" s="6"/>
     </row>
     <row r="30" ht="18" customHeight="1" spans="1:5">
       <c r="A30" s="4">
         <v>27</v>
       </c>
-      <c r="B30" s="7"/>
-      <c r="C30" s="7"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="7"/>
+      <c r="B30" s="6"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="7"/>
+      <c r="E30" s="6"/>
     </row>
     <row r="31" ht="18" customHeight="1" spans="1:5">
-      <c r="A31" s="10" t="s">
+      <c r="A31" s="11" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>